<commit_message>
Draft names for the new topics and chains; whole-corpus chart per period; numbers updated
Names drafted from top words and top motions (period 1 unchanged), to be
reviewed. The topic explorer charts shares per period instead of per
electoral term. Rubric sheet regenerated (it was not yet coded).
Documentation numbers updated to the per-period deduplication run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/docs/rubric/RUBRIC_CODING_SHEET.xlsx
+++ b/project/docs/rubric/RUBRIC_CODING_SHEET.xlsx
@@ -500,20 +500,20 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>vetenskapsråd, riksrevision, vinnova, statlig, tfhs, ämnesråd, pandemin, holdingbolag, folkmord, skolforskningsinstitut, meriteringsanställning, etikprövningsnämnd, extremism, formas, coronapandemi, jämställdhetsintegrering, lärarundantag, förberedelseskola, utvecklingsforskning, förintelse</t>
+          <t>kvinna, jämställdhet, flicka, pojke, kön, kvinnlig, manlig, kvinnoforskning, våld, mäns, genusperspektiv, forskare, norm, uppdrag, traditionell, villkor, arbete, främja, arbeta, särskilt</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2020/21 · Liberalerna · H802297 · med anledning av skr. 2019/20:199 Riksrevisionens rapport om holdingbolag vid universitet och högskolor
-1997/98 · Socialdemokraterna · GL02Ub451 · Trafikflygarhögskolan (TFHS) i Ljungbyhed
-2020/21 · Moderaterna · H802354 · med anledning av skr. 2019/20:199 Riksrevisionens rapport om holdingbolag vid universitet och högskolor
-2005/06 · Socialdemokraterna · GT02Ub475 · Trafikflyghögskolan
-1985/86 · Moderaterna · G902ub264 · Vissa fristående skolor</t>
+          <t>2004/05 · Socialdemokraterna · GS02Ub455 · Komplettering av högskoleexamina med kunskap om mäns våld mot kvinnor
+1996/97 · Socialdemokraterna · GK02Ub495 · Forskning och samhälle
+1986/87 · Socialdemokraterna · GA02Ub17 · Forskning (prop. 1986/87:80)
+2007/08 · Socialdemokraterna · GV02Ub481 · Kunskap om mäns våld mot kvinnor
+1989/90 · Socialdemokraterna · GD02Ub50 · med anledning av prop. 1989/90:90 om forskning</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -536,24 +536,24 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>forskning, universitet, svensk, forskare, utveckling, område, internationell, avancerad, satsning, lärosäte, forskarutbildning, grundnivå, vetenskaplig, högskola, land, forskarnivå, hög, resurs, samhälle, medel</t>
+          <t>adhd, hjärt, autism, diabetes, kärlsjukdom, indikator, stamning, hemundervisning, demokratiuppdrag, animation, superdator, svt, damp, dialekt, fet, specificering, hemmasittare, klassikerlista, läsutveckling, folkbokförd</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2005/06 · Folkpartiet · GT02Ub364 · EU:s forskningspolitik
-2003/04 · Folkpartiet · GR02Ub238 · EU:s forskningspolitik
-2022/23 · Moderaterna · HA021088 · Utfasning av djurförsök
-1994/95 · Miljöpartiet · GI02Ub662 · Grundforskning och forskarutbildning
-2019/20 · Miljöpartiet · H7021532 · Övergång till djurfri forskning</t>
+          <t>2005/06 · Socialdemokraterna · GT02Ub405 · Utbildning i hjärt-lungräddning
+2018/19 · Socialdemokraterna · H6022128 · Älvdalska
+2022/23 · Socialdemokraterna · HA021351 · Älvdalska
+2000/01 · Centerpartiet · GO02Ub480 · Animationens hus i Eksjö
+2008/09 · Socialdemokraterna · GW02Ub560 · Utveckling av animationen i Eksjö</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -572,24 +572,24 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>teknik, yrkeshögskola, it, teknisk, kärnämne, akademi, naturvetenskap, använda, digitalisering, naturvetenskaplig, kunskap, modern, humaniora, intresse, material, utveckla, verktyg, företagare, samhällsvetenskap, öppna</t>
+          <t>forskning, högskola, universitet, anslag, forskarutbildning, medel, förslag, verksamhet, resurs, avancerad, grundutbildning, grundnivå, område, liten, forskare, vetenskaplig, särskild, institution, professur, bedriva</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2016/17 · Socialdemokraterna · H4021138 · Idrott, matematik, fysik och kemi
-2007/08 · Socialdemokraterna · GV02Ub317 · Modern IT-teknik för att bevara skolan i glesbygden
-1988/89 · Folkpartiet · GC02Ub508 · Fortbildning av museitjänstemän
-2018/19 · Socialdemokraterna · H6022183 · Idrott för att främja intresset för teknik och naturvetenskap
-1990/91 · Moderaterna · GE02Ub643 · En natur- och kulturvetarlinje vid högskolan i Karlstad</t>
+          <t>1996/97 · Moderaterna · GK02Ub452 · Tekniskt forskningsinstitut i Göteborg
+1986/87 · Moderaterna · GA02Ub73 · Forskning (prop. 1986/87:80)
+1986/87 · Vänsterpartiet kommunisterna · GA02Ub49 · Forskning (prop. 1986/87:80)
+1991/92 · Moderaterna · GF02Ub540 · Ett råd för tvärvetenskaplig forskning
+1989/90 · Moderaterna · GD02Ub41 · med anledning av prop. 1989/90:90 om forskning</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -608,20 +608,20 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>studie, ekonomisk, student, studiemedel, system, kostnad, studera, studerande, bidrag, hög, minska, studiestöd, betala, csn, stat, höja, förslag, lån, låg, arbeta</t>
+          <t>ämne, kunskap, undervisning, elev, grundskola, ungdom, läroplan, ung, obligatorisk, gymnasieskola, lära, kränkande, hälsa, kursplan, estetisk, praktisk, fråga, hemkunskap, ingå, sexualitet</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>1998/99 · Socialdemokraterna · GM02Ub714 · Fribeloppet och studiestöd
-2006/07 · Socialdemokraterna · GU02Ub247 · Studiemedel och fribeloppet
-2013/14 · Moderaterna · H102Ub278 · Studiemedlets sammansättning och villkor
-1997/98 · Socialdemokraterna · GL02Ub713 · Inkomster under studietiden
-2013/14 · Moderaterna · H102Ub317 · Fribeloppet för studiestödet</t>
+          <t>1986/87 · Socialdemokraterna · GA02Ub225 · Översyn av läroplanen för grundskolan
+2025/26 · Centerpartiet · HD02826 · Privatekonomi för alla gymnasieelever
+1989/90 · Socialdemokraterna · GD02Ub285 · Hemkunskap och jämställdhet
+1985/86 · Folkpartiet · G902ub203 · Revidering av läroplanen för att stärka ämnet maskinskrivning
+1988/89 · Miljöpartiet · GC02Ub248 · Biologi/ekologi i gymnasieskolan</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -644,24 +644,24 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>elev, gymnasieskola, ämne, betyg, program, kunskap, grundskola, gymnasium, ungdom, kurs, lärlingsutbildning, individuell, välja, undervisning, krav, förslag, praktisk, mål, gymnasieutbildning, val</t>
+          <t>läkare, sjukvård, vård, medicinsk, hälsa, läkarutbildning, klinisk, patient, land, landsting, umeå, behov, brist, gammal, läkemedel, sjuksköterska, utbildningsplats, sjukhus, socialstyrelse, tandläkare</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>1985/86 · Folkpartiet · G902ub294 · Betygsättningen i grundskolans orienteringsämnen
-1998/99 · Socialdemokraterna · GM02Ub254 · Slutbetyg från grundskolan
-1986/87 · Folkpartiet · GA02Ub220 · Betygssystemet i grundskolan
-1987/88 · Folkpartiet · GB02Ub212 · om betygssystemet i grundskolan Mot.
-1987/88 · Folkpartiet · GB02Ub211 · om utökat praktiskt tillval i grundskolan</t>
+          <t>1996/97 · Socialdemokraterna · GK02Ub460 · Läkarutbildningen vid Umeå universitet
+1996/97 · Centerpartiet · GK02Ub474 · Utökad läkarutbildning i Umeå
+1986/87 · Centerpartiet · GA02Ub631 · Ökad läkarutbildning i Umeå
+2008/09 · Socialdemokraterna · GW02Ub211 · Utökad läkar- och tandläkarutbildning i Norrland
+2007/08 · Socialdemokraterna · GV02Ub275 · Utökad läkar- och tandläkarutbildning i Norrland</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -680,24 +680,24 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>kommun, elev, fristående, kommunal, friskola, förälder, verksamhet, välja, skolverk, skollag, likvärdig, skolväsende, bidrag, barn, grundskola, behov, offentlig, resurs, statsbidrag, tillsyn</t>
+          <t>gymnasieskola, program, elev, kurs, yrkesutbildning, gymnasium, kunskap, krav, ungdom, behov, arbetsliv, studie, hög, lärlingsutbildning, arbetsmarknad, gymnasieutbildning, förslag, behörighet, välja, lärande</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1988/89 · Moderaterna · GC02Ub279 · Bidraget till fristående skolor
-2008/09 · Socialdemokraterna · GW02Ub356 · Fristående skolors elevansvar
-1990/91 · Moderaterna · GE02Ub8 · med anledning av prop. 1990/91:18 Ansvaret för skolan
-2006/07 · Moderaterna · GU02Ub292 · Skolskjutsar
-2007/08 · Socialdemokraterna · GV02Ub398 · Kommuners beslutanderätt vid etablering av friskolor</t>
+          <t>1989/90 · Socialdemokraterna · GD02Ub229 · Reformering av yrkesutbildning
+2010/11 · Socialdemokraterna · GY02Ub457 · Behörighet till högskolestudier
+2016/17 · Sverigedemokraterna · H4021379 · Återinföra tvåårigt gymnasium för praktiska och estetiska linjer med möjlighet till förlängning
+2000/01 · Moderaterna · GO02Ub209 · Funktionshindrade ungdomars valfrihet
+1992/93 · Folkpartiet · GG02Ub470 · Gymnasiestudierna</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -716,20 +716,20 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>anslag, högskola, förslag, medel, resurs, liten, särskild, verksamhet, budgetår, grundutbildning, forskning, bidrag, anvisa, anslå, universitet, ytterlig, medelstor, minska, åtgärd, utveckling</t>
+          <t>forskning, utveckling, svensk, lärosäte, hög, internationell, kvalitet, stärka, nationell, land, utveckla, forskare, område, satsning, näringsliv, samhälle, kunskap, samverkan, företag, yrkeshögskola</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1996/97 · Moderaterna · GK02Ub452 · Tekniskt forskningsinstitut i Göteborg
-1992/93 · Centerpartiet · GG02Ub124 · med anledning av prop. 1992/93:170 Forskning för kunskap och framsteg
-1989/90 · Folkpartiet · GD02Ub150 · med anledning av prop. 1989/90 om forskning
-1989/90 · Folkpartiet · GD02Ub73 · med anledning av prop. 1989/90:90 om forskning
-1986/87 · Moderaterna · GA02Ub648 · Högskolan i Växjö</t>
+          <t>2011/12 · Moderaterna · GZ02Ub333 · En svensk klimatforskningssatellit
+2010/11 · Moderaterna · GY02Ub332 · Forskning om IT och ny teknik
+2012/13 · Socialdemokraterna · H002Ub418 · Forskning för att utveckla och miljöanpassa flyget
+2022/23 · Kristdemokraterna · HA021363 · Effektmål för innovationer
+2014/15 · Moderaterna · H202152 · Nya generationens kärnkraft</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -752,24 +752,24 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>läkare, läkarutbildning, land, fn, utbildningsplats, läkemedel, plats, sjukvård, universitetskanslersämbete, fred, utöka, mänsklig, at, tal, landsting, rättighet, behov, utbilda, brist, avtal</t>
+          <t>åtgärd, lag, skolverk, lärare, uppdrag, rektor, problem, myndighet, införa, förslag, person, regel, krav, brist, trakasseri, tydlig, utreda, anställning, bedömning, allvarlig</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>1989/90 · Centerpartiet · GD02Ub562 · Receptarie- och apotekareutbildning
-1988/89 · Centerpartiet · GC02Ub645 · Ökad receptarie- och apotekarutbildning
-1988/89 · Moderaterna · GC02Ub659 · Receptarie- och apotekareutbildning
-1988/89 · Folkpartiet · GC02Ub565 · Utökad receptarie- och apotekarutbildning
-1989/90 · Socialdemokraterna · GD02Ub576 · Receptarie- och apotekarutbildningen</t>
+          <t>2024/25 · Moderaterna · HC021831 · Översyn av registerutdrag
+2021/22 · Moderaterna · H9022802 · Rektorsutbildningen
+1988/89 · Folkpartiet · GC02Ub237 · Lärares uppsägningstid
+1986/87 · Moderaterna · GA02Ub214 · Ersättare för lärare som förordnats som skolledare
+2008/09 · Socialdemokraterna · GW02Ub409 · Utöka lagen om registerkontroll av personal inom förskoleverksamhet, skola och skolbarnsomsorg</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -788,24 +788,24 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>hälsa, kunskap, sjukdom, mat, hemkunskap, ämne, psykisk, dålig, kost, arbetsmiljö, skolhälsovård, drabba, äta, människa, betydelse, medicinsk, konsument, ungdom, samband, konsumentkunskap</t>
+          <t>kommun, fristående, kommunal, skolverk, verksamhet, bidrag, förslag, stat, kostnad, huvudman, statsbidrag, välja, skolväsende, statlig, offentlig, ekonomisk, tillsyn, likvärdig, bedriva, enskild</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>1988/89 · Folkpartiet · GC02Ub640 · Undervisningen i klinisk mykologi
-1988/89 · Folkpartiet · GC02Ub642 · Forskningen i medicinsk mykologi
-2005/06 · Centerpartiet · GT02Ub392 · Medicinsk forskning för bättre hälsa
-2001/02 · Moderaterna · GP02Ub262 · Grundforskningen om fibromyalgi
-1989/90 · Folkpartiet · GD02Ub531 · Utökad undervisning i klinisk mykologi</t>
+          <t>1989/90 · Folkpartiet · GD02Ub283 · Statsbidraget till estniska skolan
+1995/96 · Socialdemokraterna · GJ02Ub37 · med anledning av prop. 1995/96:200 Fristående skolor m.m.
+1989/90 · Centerpartiet · GD02Ub215 · Statsbidraget för lärarlöner inom grundskolan
+1986/87 · Folkpartiet · GA02Ub58 · Forskning (prop. 1986/87:80)
+1994/95 · Socialdemokraterna · GI02Ub352 · Lundsbergs skola</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -824,24 +824,24 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>sfi, invandrare, svensk, nyanländ, undervisning, timme, svenska, arbetsmarknad, jobb, körkort, kommun, svenskundervisning, utländsk, samhälle, arbete, erbjuda, flykting, undervisningstid, person, krav</t>
+          <t>samhälle, människa, kunskap, svensk, land, utveckling, arbete, social, problem, uppgift, ansvar, fråga, form, politisk, utveckla, område, använda, individ, intresse, betydelse</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>1986/87 · Folkpartiet · GA02Ub272 · Koncentrerad svenskundervisning för invandrare
-1989/90 · Folkpartiet · GD02Ub17 · med anledning av prop. 1989/90:102 om reformerad svenskundervisning för vuxna invandrare
-1988/89 · Socialdemokraterna · GC02Ub256 · Ökade resurser för grundvux
-1987/88 · Folkpartiet · GB02Ub207 · om koncentrerad SFI-undervisning
-1986/87 · Socialdemokraterna · GA02Ub238 · Grundvux för invandrare</t>
+          <t>2001/02 · Socialdemokraterna · GP02Ub503 · Information i skolan från politiska partier
+2010/11 · Socialdemokraterna · GY02Ub247 · Kolonialismen i historieundervisningen
+1988/89 · Socialdemokraterna · GC02Ub586 · Folklivsforskningen
+2015/16 · Socialdemokraterna · H302834 · Motverkande av rasism och diskriminering i skolväsendet
+2000/01 · Kristdemokraterna · GO02Ub283 · Ungdomars delaktighet i samhällets demokratiska processer</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -860,16 +860,16 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>barn, förälder, ungdom, ung, social, samhälle, problem, vuxen, sexuell, familj, liv, arbete, person, utsatt, funktionsnedsättning, grupp, situation, svår, rättighet, miljö</t>
+          <t>land, arbetsmarknad, hög, företag, jobb, ung, kompetens, person, människa, tillgång, behov, erbjuda, arbete, universitet, kompetensutveckling, it, satsning, arbeta, utveckla, arbetskraft</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>1989/90 · Folkpartiet · GD02Ub287 · Undervisningen i teckenspråk
-1989/90 · Socialdemokraterna · GD02Ub253 · Undervisningen i teckenspråk
-2024/25 · Moderaterna · HC021121 · Obligatorisk undervisning om sexuella övergrepp
-2007/08 · Socialdemokraterna · GV02Ub372 · Föräldrars möjlighet till delaktighet i skola och förskola
-2019/20 · Moderaterna · H7021950 · Elevhälsans hälsosamtal</t>
+          <t>2019/20 · Socialdemokraterna · H7021829 · Kompetensutveckling som möter teknikutveckling och en ökad digitalisering
+2015/16 · Sverigedemokraterna · H3021446 · Företagsdag på högstadiet och gymnasiet
+2002/03 · Socialdemokraterna · GQ02Ub447 · Vuxenutbildning för arbetslösa
+2010/11 · Moderaterna · GY02Ub330 · IT-utbildningar på högskolan och för småföretagare
+2014/15 · Moderaterna · H2021784 · Ung företagsamhet</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
@@ -896,24 +896,24 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>universitet, göteborg, umeå, lund, örebro, stockholm, institution, uppsala, professur, land, verksamhet, bedriva, fakultet, centrum, institut, inrätta, område, västsverige, tjänst, samarbete</t>
+          <t>stockholm, uppsala, teologisk, lokal, södertälje, anläggning, verksamhet, hyra, centrum, campus, statlig, bolag, ess, hls, stiftelse, tfhs, ägare, lokalkostnad, oseriös, byggande</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>1986/87 · Folkpartiet · GA02Ub78 · Forskning (prop. 1986/87:80)
-2012/13 · Moderaterna · H002Ub267 · Lunds universitets historiska museum
-1996/97 · Socialdemokraterna · GK02Ub439 · Examinationsrätt till apotekarexamen vid Göteborgs universitet
-1989/90 · Folkpartiet · GD02Ub75 · med anledning av prop. 1989/90:90 om forskning
-1985/86 · Folkpartiet · G902ub570 · Universitetsbiblioteket i Lund</t>
+          <t>1985/86 · Moderaterna · G902ub526 · Nya lokaler för landsarkivet i Uppsala
+1987/88 · Socialdemokraterna · GB02Ub644 · om lokalisering till Södertälje av högskolan för lärarutbildning
+1987/88 · Centerpartiet · GB02Ub729 · om lokalisering av HLS till Södertälje
+1986/87 · Centerpartiet · GA02Ub502 · Utbyggnaden av Vadstena slott
+1985/86 · Socialdemokraterna · G902ub557 · Ombyggnad av lokaler för högskolan i Skövde</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -932,16 +932,16 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>kvinna, kunskap, samhälle, människa, jämställdhet, flicka, arbete, pojke, utveckling, område, demokrati, kön, fråga, social, demokratisk, utveckla, handla, kvinnlig, perspektiv, arbeta</t>
+          <t>lärare, lärarutbildning, pedagogisk, undervisning, ämne, fortbildning, läraryrke, kunskap, kompetens, undervisa, behörig, krav, värdegrund, kvalitet, grundskola, religiös, inriktning, yrke, kristen, brist</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2005/06 · Socialdemokraterna · GT02Ub473 · Jämställdhet i undervisningen
-2008/09 · Socialdemokraterna · GW02Ub276 · Jämställdhet i högre utbildning
-1989/90 · Folkpartiet · GD02Ub209 · Ämnet maskinskrivning i grundskolan
-2000/01 · Kristdemokraterna · GO02Ub293 · Manligt maktutövande
-1990/91 · Folkpartiet · GE02Ub276 · Maskinskrivning som ämnesbeteckning</t>
+          <t>1988/89 · Centerpartiet · GC02Ub311 · Religionskunskap i skolundervisningen
+1990/91 · Moderaterna · GE02Ub815 · Utbildning av lärare i religionskunskap
+2011/12 · Socialdemokraterna · GZ02Ub402 · Introduktionsår för lärare
+1988/89 · Folkpartiet · GC02Ub573 · Den pedagogiska utbildningen för lärare vid universitet och högskolor
+1987/88 · Socialdemokraterna · GB02Ub509 · om behörighetsgrunderna för tjänst som högskolelektor</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
@@ -968,16 +968,16 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>förslag, verksamhet, uppgift, ansvar, politisk, krav, enskild, återkomma, lokal, fråga, bedömning, problem, princip, risk, lagstiftning, konsekvens, frihet, organisation, ange, lägga</t>
+          <t>mat, läromedel, allians, äta, ungdom, skolmat, skolsköterska, bok, elev, dålig, hälsa, barnkonvention, tjej, kost, skolmåltid, barn, undersökning, servera, frukost, måltid</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>1985/86 · Moderaterna · G902ub578 · Besvärsrätten inom högskoleområdet
-2008/09 · Moderaterna · GW02Ub429 · Kår- och nationsobligatoriets avskaffande
-2006/07 · Socialdemokraterna · GU02Ub341 · Kårobligatoriet
-1990/91 · Socialdemokraterna · GE02Ub571 · Avveckling av kårobligatoriet
-2003/04 · Miljöpartiet · GR02Ub329 · Kårobligatoriet</t>
+          <t>1989/90 · Centerpartiet · GD02Ub205 · Skolmåltiderna
+1988/89 · Centerpartiet · GC02Ub219 · Skolmåltider
+2005/06 · Socialdemokraterna · GT02Ub561 · Gratis skolmat i gymnasiet
+2019/20 · Sverigedemokraterna · H702724 · Säkra tallriksmodellen i skolan
+2004/05 · Socialdemokraterna · GS02Ub484 · Lagstadgad skolmat</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
@@ -1004,16 +1004,16 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>nationell, uppdrag, kvalitet, myndighet, tydlig, stärka, skolverk, stat, hållbar, brist, fokus, utredning, ansvar, rapport, granskning, arbete, uppföljning, finansiering, utvärdering, resultat</t>
+          <t>språk, svensk, undervisning, svenska, invandrare, sfi, modersmål, nyanländ, kommun, samhälle, timme, land, hemspråksundervisning, andraspråk, diskriminering, lära, kultur, svenskundervisning, finsk, erbjuda</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2021/22 · Moderaterna · H9021866 · Central rättning av centrala prov
-2025/26 · Socialdemokraterna · HD023970 · med anledning av skr. 2025/26:166 Riksrevisionens rapport om utbildning på vetenskaplig grund
-2011/12 · Moderaterna · GZ02Ub432 · Validering av utbildningar från andra länder
-2019/20 · Moderaterna · H70252 · med anledning av skr. 2018/19:144 Riksrevisionens rapport om Skolinspektionens uppföljning av brister i skolor
-2010/11 · Vänsterpartiet · GY02Ub283 · Utvärdering av skolans styrning och finansiering</t>
+          <t>1986/87 · Folkpartiet · GA02Ub272 · Koncentrerad svenskundervisning för invandrare
+2008/09 · Socialdemokraterna · GW02Ub450 · Svenska för invandrare
+1989/90 · Folkpartiet · GD02Ub1 · med anledning av prop. 1989/90:25 med förslag om tilläggsbudget I till statsbudgeten för budgetåret 1989/90
+1987/88 · Folkpartiet · GB02Ub207 · om koncentrerad SFI-undervisning
+1988/89 · Socialdemokraterna · GC02Ub329 · Undervisningen i svenska för vuxna invandrare m.m.</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -1040,20 +1040,20 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>vuxenutbildning, behov, arbetsmarknad, lärande, folkhögskola, människa, yrkesutbildning, samhälle, arbetsliv, kunskap, komvux, vuxen, kompetens, livslång, kvalificerad, arbete, utveckla, folkbildning, studieförbund, jobb</t>
+          <t>elev, lärare, grundskola, betyg, undervisning, nationell, kunskap, stöd, mål, friskola, förälder, nå, årskurs, ansvar, resultat, särskild, prov, tydlig, skollag, läsa</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2006/07 · Socialdemokraterna · GU02Ub374 · Studiefinansiering
-2006/07 · Socialdemokraterna · GU02Ub373 · Stöd till kommuner för att bedriva vuxenutbildning
-2007/08 · Socialdemokraterna · GV02Ub410 · Vuxenutbildningen
-2006/07 · Socialdemokraterna · GU02Ub229 · Vuxenutbildning
-2004/05 · Socialdemokraterna · GS02Ub381 · Vuxenutbildningen</t>
+          <t>2020/21 · Socialdemokraterna · H8021572 · Åtgärder för rättvis betygsättning och att motverka betygsinflation
+2008/09 · Socialdemokraterna · GW02Ub380 · Ytterligare satsningar på grundskolan
+2011/12 · Moderaterna · GZ02Ub462 · Central rättning av nationella prov
+2014/15 · Moderaterna · H2021535 · Central rättning av nationella prov
+2001/02 · Kristdemokraterna · GP02Ub342 · Betyg</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -1076,24 +1076,24 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>elev, lärare, undervisning, kunskap, grundskola, lärarutbildning, mobbning, stöd, rektor, ansvar, läsa, nå, mål, arbete, tydlig, årskurs, införa, skolverk, prov, lära</t>
+          <t>behov, stöd, särskild, särskola, funktionshind, barngrupp, kompetens, specialskola, grupp, malmö, handikapp, institut, barn, elev, personal, döv, utredning, brist, kommun, land</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2024/25 · Socialdemokraterna · HC021761 · Hjälpmedel vid nationella prov för elever med dyslexi
-1998/99 · Moderaterna · GM02Ub212 · Stöd till elever med läs- och skrivsvårigheter
-2001/02 · Centerpartiet · GP02Ub418 · Dyslexi
-2013/14 · Moderaterna · H102Ub281 · Behovet av speciallärare
-2019/20 · Moderaterna · H7021627 · Utöka antalet skoldagar i svensk skola</t>
+          <t>1991/92 · Folkpartiet · GF02Ub59 · med anledning av prop. 1991/92:94 Ändrat huvudmannaskap för särskolan och särvux m.m.
+1991/92 · Socialdemokraterna · GF02Ub303 · Regionala resurscentra för elever med autism
+1991/92 · Centerpartiet · GF02Ub282 · Regionala resurscentra för elever med autism
+1994/95 · Centerpartiet · GI02Ub319 · Statens institut för handikappfrågor i skolan
+1990/91 · Vänsterpartiet · GE02Ub713 · Psykoterapiutbildning för psykologer</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -1112,24 +1112,24 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>nivå, konstnärlig, mälardalens, malmö, musik, borås, kultur, stockholm, musikhögskola, verksamhet, konsthögskola, samisk, statlig, konstfack, stöd, design, hög, film, utanförskapsområde, musikskola</t>
+          <t>social, vård, landsting, omsorg, vårdutbildning, vårdhögskola, huvudmannaskap, sjuksköterska, arbete, statlig, personal, hälsa, omvårdnad, hälsofrämjande, kommunal, äldreomsorg, förtryck, ledd, undersköterska, bostadsbidrag</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>1989/90 · Folkpartiet · GD02Ub697 · En konsthögskola i Malmö
-1988/89 · Moderaterna · GC02Ub281 · Konstskolan BASIS
-1991/92 · Folkpartiet · GF02Ub206 · Utbildningen av yrkesvalslärare
-1988/89 · Folkpartiet · GC02Ub816 · Utbildningen av yrkesvalslärare
-1992/93 · Folkpartiet · GG02Ub34 · med anledning av prop. 1992/93:169 Högre utbildning för ökad kompetens</t>
+          <t>1986/87 · Folkpartiet · GA02Ub574 · Alternativ i sjuksköterskeutbildningen
+1989/90 · Moderaterna · GD02Ub621 · Utbildningsfrågor inom hälso- och sjukvården
+1987/88 · Moderaterna · GB02Ub808 · om utbildningsfrågor inom hälso- och sjukvården
+1988/89 · Moderaterna · GC02Ub810 · Utbildningsfrågor inom hälso- och sjukvården
+1994/95 · Centerpartiet · GI02Ub619 · Landstingskommunal vårdhögskola</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -1148,16 +1148,16 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>idrott, fysisk, aktivitet, hälsa, fritid, rörelse, ämne, friluftsliv, timme, ungdom, aktiv, trafik, idrottsämne, utveckling, idrottshögskola, skog, idrottsrörelse, anläggning, homo, träning</t>
+          <t>lärcentrum, rekryteringsbidrag, hbt, homosexuell, bisexuell, transperson, östersjön, marin, lärcentra, koncern, utförare, hav, heterosexuell, skl, gesällprov, homosexualitet, nitus, retorik, teknikcollege, bisexualitet</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2016/17 · Moderaterna · H402495 · Mer rörelse och idrott i skolan
-1985/86 · Centerpartiet · G902ub610 · Behovet av en särskild idrottshögskola
-2000/01 · Moderaterna · GO02Ub268 · Idrottstimmar i skolan
-1992/93 · Centerpartiet · GG02Ub442 · Idrottsämnet i skolan
-2001/02 · Moderaterna · GP02Ub310 · Idrottsämnet</t>
+          <t>2001/02 · Socialdemokraterna · GP02Ub542 · Homo-, bisexuella och transpersoner i skolan
+1999/2000 · Socialdemokraterna · GN02Ub280 · Feminism i skolans läroplan
+1988/89 · Moderaterna · GC02Ub564 · Lokalisering av ett Östersjölaboratorium i Karlskrona
+2020/21 · Moderaterna · H802354 · med anledning av skr. 2019/20:199 Riksrevisionens rapport om holdingbolag vid universitet och högskolor
+2008/09 · Socialdemokraterna · GW02Ub326 · Vuxenstuderandes rätt till ekonomisk ersättning</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -1184,20 +1184,20 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>kränkning, ky, utbildningsvetenskaplig, vfu, skolavslutning, rektorsutbildning, otrygg, kill, avstängning, värdegrundsarbete, åka, mobilitet, upplägg, förtydligad, anmälningsplikt, spetsforskning, utbildningsvetenskap, utförare, kvalitetsredovisning, unescoråd</t>
+          <t>barn, förskola, förälder, kommun, verksamhet, personal, barnomsorg, behov, pedagogisk, skolverk, kvalitet, fritidshem, familj, arbeta, erbjuda, utveckling, liten, förskollärare, stöd, omsorg</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>1986/87 · Socialdemokraterna · GA02Ub228 · Skolavslutning på lördagar
-1999/2000 · Socialdemokraterna · GN02Ub280 · Feminism i skolans läroplan
-2019/20 · Kristdemokraterna · H702295 · Skolavslutning med konfessionella inslag i kyrkolokaler
-2004/05 · Moderaterna · GS02Ub204 · Kvalificerad yrkesutbildning
-1985/86 · Socialdemokraterna · G902ub590 · Lokaliseringen till Mälardalen av en ny superdator</t>
+          <t>2010/11 · Socialdemokraterna · GY02Ub358 · Barns rätt till skola, barnomsorg och fritis
+2013/14 · Socialdemokraterna · H102Ub544 · Alla barns rätt till förskola
+2013/14 · Socialdemokraterna · H102Ub558 · Barnomsorg på heltid
+2010/11 · Socialdemokraterna · GY02Ub393 · En bra förskola för våra barn
+2006/07 · Socialdemokraterna · GU02Ub411 · Resurser till fritidsverksamheterna</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -1220,24 +1220,24 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>svensk, språk, land, svenska, undervisning, modersmål, internationell, teckenspråk, nordisk, engelsk, kultur, andraspråk, läsa, finsk, kunskap, värld, tala, minoritet, utomlands, minoritetsspråk</t>
+          <t>högskola, län, region, plats, utveckling, teknisk, hög, behov, linje, universitet, regional, lokal, land, högskoleutbildning, resurs, liten, område, ytterlig, näringsliv, kurs</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>1988/89 · Folkpartiet · GC02Ub541 · En professur i turkiska språk och turkisk kultur
-1989/90 · Folkpartiet · GD02Ub70 · med anledning av prop. 1989/90:90 om forskning
-1992/93 · Folkpartiet · GG02Ub602 · Forskning i turkiska språken och kulturen
-2017/18 · Socialdemokraterna · H5022174 · Tyska språket i skolan
-2007/08 · Folkpartiet · GV02Ub475 · Hillelskolan</t>
+          <t>1989/90 · Moderaterna · GD02Ub740 · Dimensionering av vissa utbildningslinjer vid högskolan i Gävle—Sandviken
+1988/89 · Socialdemokraterna · GC02Ub606 · Högskolan i Karlskrona/Ronneby
+1986/87 · Socialdemokraterna · GA02Ub610 · Utbildningen i småföretagsekonomi vid högskolan i Falun/Borlänge
+1990/91 · Socialdemokraterna · GE02Ub663 · Ingenjörsutbildningen vid högskolan i Karlskrona-Ronneby
+1986/87 · Centerpartiet · GA02Ub556 · Utbildningsväsendet och den regionala</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -1256,24 +1256,24 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>högskola, län, jönköping, gävle, kristianstad, sandviken, halmstad, gävleborg, yrkesvux, låg, tilldela, söktryck, utbildningsnivå, försäkringskassa, uppsala, rike, gymnastik, spetsutbildning, kommun, ungdom</t>
+          <t>förskoleklass, validering, kvalitetsinstitut, lovskola, skolavslutning, simundervisning, svensk, transparent, lära, simkunnighet, otrygg, simma, arbetsmiljöverk, förort, kärnämneskurs, implementera, kristdemokrat, lågstadium, kunskapskontrakt, skoluniform</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>1990/91 · Folkpartiet · GE02Ub651 · Ekonomlinjen vid högskolan i Jönköping
-1987/88 · Folkpartiet · GB02Ub721 · om ekonomlinjen vid högskolan i Jönköping
-1988/89 · Moderaterna · GC02Ub722 · Ekonomutbildningen vid högskolan i Kristianstad
-1988/89 · Centerpartiet · GC02Ub557 · Ekonomiutbildningen vid högskolan i Kristianstad
-1992/93 · Socialdemokraterna · GG02Ub146 · med anledning av prop. 1992/93:170 Forskning för kunskap och framsteg</t>
+          <t>2003/04 · Socialdemokraterna · GR02Ub432 · Simundervisning i skolan
+1994/95 · Vänsterpartiet · GI02Ub363 · Simundervisningen
+2002/03 · Socialdemokraterna · GQ02Ub436 · Barns simundervisning i skolan
+2013/14 · Socialdemokraterna · H102Ub543 · Vikten av simkunnighet och små barns rätt till vattenvana
+2006/07 · Socialdemokraterna · GU02Ub384 · Simundervisning</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1292,20 +1292,20 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>högskola, linje, plats, behov, teknisk, län, kurs, högskoleutbildning, område, inriktning, lokal, poäng, studerande, ytterlig, lärarutbildning, utveckling, skövde, kommun, karlstad, resurs</t>
+          <t>student, högskola, hög, studie, förslag, studerande, studiemedel, system, anslag, lärosäte, studera, ekonomisk, minska, studiestöd, bidrag, enskild, csn, höja, regel, kvalitet</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>1987/88 · Folkpartiet · GB02Ub574 · om mellaningenjörsutbildning i Borås
-1988/89 · Centerpartiet · GC02Ub23 · med anledning av prop. 1988/89:90 om
-1989/90 · Centerpartiet · GD02Ub632 · Ingenjörsutbildning till Ljungby
-1989/90 · Moderaterna · GD02Ub740 · Dimensionering av vissa utbildningslinjer vid högskolan i Gävle—Sandviken
-1989/90 · Moderaterna · GD02Ub525 · Förskollärarutbildning vid högskolan i Borås</t>
+          <t>2011/12 · Moderaterna · GZ02Ub269 · Fribeloppets avskaffande
+2011/12 · Kristdemokraterna · GZ02Ub313 · Slopat fribelopp i studiemedlet
+2013/14 · Moderaterna · H102Ub278 · Studiemedlets sammansättning och villkor
+2008/09 · Moderaterna · GW02Ub429 · Kår- och nationsobligatoriets avskaffande
+2002/03 · Moderaterna · GQ02Ub237 · Avskaffande av fribeloppet</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -1328,16 +1328,16 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>företag, land, hög, utveckling, region, näringsliv, regional, utveckla, liten, högskola, satsning, samarbete, kommun, behov, tillgång, samverkan, lokal, betydelse, tillväxt, kompetens</t>
+          <t>entreprenörskap, kalmar, bibliotek, företagande, turism, starta, kooperativ, natt, mus, ekonomi, samling, linnéuniversitetet, skoglig, södra, yh, näring, museum, hotell, rekreation, arkiv</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>1988/89 · Centerpartiet · GC02Ub599 · En högskola i Kiruna
-1989/90 · Centerpartiet · GD02Ub514 · Högskola till Kiruna
-2013/14 · Socialdemokraterna · H102Ub270 · Ung företagsamhet
-1999/2000 · Socialdemokraterna · GN02Ub470 · Rymdhögskola i Kiruna
-2002/03 · Centerpartiet · GQ02Ub257 · Kvalificerad yrkesutbildning</t>
+          <t>1988/89 · Folkpartiet · GC02Ub508 · Fortbildning av museitjänstemän
+1987/88 · Folkpartiet · GB02Ub597 · om fortbildning av museitjänstemän
+1986/87 · Folkpartiet · GA02Ub647 · Lokal för utställningar inom Kungliga biblioteket
+1991/92 · Socialdemokraterna · GF02Ub438 · Mikrofilmning av affischer
+2014/15 · Moderaterna · H202268 · Lunds universitets historiska museum</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -1364,24 +1364,24 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>elev, behov, särskola, funktionshind, stöd, specialskola, särskild, läromedel, handikapp, funktionshindrad, döv, undervisning, anpassad, synskadad, handikappad, hjälpmedel, grundskola, skolform, skolgång, tillgång</t>
+          <t>psykisk, sjukdom, arbetsmiljö, problem, ohälsa, kränkning, drabba, behandling, ung, hälsa, förebyggande, person, fysisk, tidig, arbete, dålig, risk, vanlig, hjälp, åtgärd</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>1985/86 · Vänsterpartiet kommunisterna · G902ub282 · Rikscentralerna för pedagogiska hjälpmedel för handikappade
-1992/93 · Folkpartiet · GG02Ub468 · Läromedel för begåvningshandikappade elever
-1987/88 · Folkpartiet · GB02Ub282 · om läromedelsförsörjningen för synskadade elever
-1987/88 · Moderaterna · GB02Ub336 · om läromedel till synskadade elever
-1987/88 · Socialdemokraterna · GB02Ub226 · om läromedelsförsörjningen för synskadade</t>
+          <t>2025/26 · Centerpartiet · HD021169 · Prioritering av forskning om behandling av cytostatikainducerad neuropati
+1988/89 · Socialdemokraterna · GC02Ub238 · Arbetsmiljöutbildning
+2001/02 · Socialdemokraterna · GP02Ub527 · Hörselskador i barnomsorg och skola
+2018/19 · Centerpartiet · H6022344 · Inför psykiska hälsokontroller för skolungdomar
+2003/04 · Socialdemokraterna · GR02Ub501 · Forskning om migrän</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1400,24 +1400,24 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>narkotika, hbt, ant, fråga, undervisning, bisexuell, barnkunskap, indikator, verk, gymnasieår, bruk, röka, ja, mental, tragedi, folkhälsoinstitut, länsskolnamnd, pilot, ämnesplan, bisexualitet</t>
+          <t>göteborg, skövde, konstnärlig, västsverige, skaraborg, region, fjärrundervisning, trollhättan, område, uddevalla, väst, ai, design, västsvensk, industri, livsmedelsindustri, lärande, världsledande, kultur, kompetens</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>1993/94 · Folkpartiet · GH02Ub620 · ANT-undervisningen för lärare
-1990/91 · Socialdemokraterna · GE02Ub818 · Undervisning i skolan om alkohol, narkotika och tobak (ANT)
-1991/92 · Centerpartiet · GF02Ub26 · med anledning av prop. 1991/92:75 Lärarutbildning m.m.
-2002/03 · Socialdemokraterna · GQ02Ub544 · HBT-frågor i undervisningsväsendet
-2013/14 · Socialdemokraterna · H102Ub368 · Kompetens om hbt-frågor inom utbildningssystemet och statliga myndigheter</t>
+          <t>1989/90 · Centerpartiet · GD02Ub562 · Receptarie- och apotekareutbildning
+1988/89 · Centerpartiet · GC02Ub645 · Ökad receptarie- och apotekarutbildning
+1989/90 · Socialdemokraterna · GD02Ub576 · Receptarie- och apotekarutbildningen
+1988/89 · Moderaterna · GC02Ub659 · Receptarie- och apotekareutbildning
+1988/89 · Folkpartiet · GC02Ub565 · Utökad receptarie- och apotekarutbildning</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1436,20 +1436,20 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>skolinspektion, huvudman, elevhälsa, utreda, alliansregering, tillstånd, befogenhet, neuropsykiatrisk, huvudmannaskap, samtycke, lovskola, kpu, granska, lärarlön, skolkoncern, branschskola, etikprövning, person, adhd, simundervisning</t>
+          <t>skolinspektion, elevhälsa, alkohol, handlingsplan, tuff, ant, fetma, tobak, dans, utanförskap, mobiltelefon, studentexamen, yrkesvägled, otillåten, world, ogiltig, yrkande, fritidsprogram, röka, syndrom</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2006/07 · Socialdemokraterna · GU02Ub384 · Simundervisning
-2002/03 · Socialdemokraterna · GQ02Ub436 · Barns simundervisning i skolan
-2003/04 · Socialdemokraterna · GR02Ub432 · Simundervisning i skolan
-1994/95 · Vänsterpartiet · GI02Ub363 · Simundervisningen
-2024/25 · Kristdemokraterna · HC021133 · Registerkontroll inom skola och barnomsorg</t>
+          <t>1988/89 · Centerpartiet · GC02Ub273 · Obligatorisk dansundervisning i grundskolan
+1988/89 · Socialdemokraterna · GC02Ub681 · Folkdanslinje på Danshögskolan
+1992/93 · Folkpartiet · GG02Ub683 · Utbildning för sjukvårdspersonal om alkohol
+1990/91 · Socialdemokraterna · GE02Ub818 · Undervisning i skolan om alkohol, narkotika och tobak (ANT)
+1991/92 · Centerpartiet · GF02Ub26 · med anledning av prop. 1991/92:75 Lärarutbildning m.m.</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
@@ -1472,24 +1472,24 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>läroplan, ämne, undervisning, samhälle, människa, värde, värdegrund, religiös, våld, etisk, värdering, kristen, religion, etik, fråga, svensk, konfessionell, kunskap, respekt, sexualitet</t>
+          <t>mälardalens, riksrevision, etisk, djur, djurförsök, alternativ, fn, metod, material, konvention, yrkesexam, fred, universitetskanslersämbete, rekommendation, hantverkare, hantverk, konflikt, gammal, institution, levande</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>1996/97 · Socialdemokraterna · GK02Ub218 · En mångkulturell skola m.m.
-1988/89 · Centerpartiet · GC02Ub311 · Religionskunskap i skolundervisningen
-2007/08 · Socialdemokraterna · GV02Ub285 · Skolans värdegrund
-2009/10 · Socialdemokraterna · GX02Ub280 · Ersättande av begreppet kristen tradition i läroplanen
-1994/95 · Moderaterna · GI02Ub303 · Etikundervisning</t>
+          <t>1988/89 · Folkpartiet · GC02Ub306 · Djurförsök i skolan
+1987/88 · Folkpartiet · GB02Ub634 · om djurförsöken i utbildningen
+1989/90 · Folkpartiet · GD02Ub673 · Djurhuset vid Sahlgrenska sjukhuset
+1988/89 · Folkpartiet · GC02Ub733 · Djurhuset vid Sahlgrenska sjukhuset
+1989/90 · Centerpartiet · GD02Ub663 · Stiftelsen Skånehantverk i Landskrona</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -1508,24 +1508,24 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>vård, behov, landsting, sjukvård, hälsa, ohälsa, sjuksköterska, patient, personal, medicinsk, klinisk, yrke, gammal, brist, kompetens, vårdutbildning, krav, omsorg, vårdhögskola, arbeta</t>
+          <t>nivå, universitet, forskarnivå, lund, linköping, nordisk, högskolebehörighet, poäng, svensk, skåne, kunglig, kristianstad, beräknad, norrköping, norden, danmark, sjukgymnast, historia, studie, norge</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>1986/87 · Folkpartiet · GA02Ub574 · Alternativ i sjuksköterskeutbildningen
-1989/90 · Socialdemokraterna · GD02Ub606 · Laboratorieassistentutbildningen
-1989/90 · Folkpartiet · GD02Ub736 · Laboratorieassistentutbildningens anpassning till Norden och EG
-1986/87 · Folkpartiet · GA02Ub620 · Antagningen till psykoterapiutbildning
-1993/94 · Moderaterna · GH02Ub666 · Geriatrikutbildning för vårdpersonal</t>
+          <t>1993/94 · Kristen demokratisk samling · GH02Ub698 · Master of Science-examen vid de tekniska högskolorna
+1990/91 · Miljöpartiet · GE02Ub709 · Juristlinjen vid universitetet i Göteborg
+1988/89 · Vänsterpartiet kommunisterna · GC02Ub695 · Högskoleutbildning av optiker vid universitetet i Linköping
+1988/89 · Centerpartiet · GC02Ub572 · Utökad sjukgymnastutbildning
+1987/88 · Centerpartiet · GB02Ub502 · om sjukgymnastutbildning i Kristianstads län</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -1544,16 +1544,16 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>student, högskola, hög, universitet, lärosäte, kvalitet, lärare, akademisk, studie, krav, kurs, person, exam, studerande, kompetens, digital, högskoleutbildning, rekrytering, högskoleverk, utländsk</t>
+          <t>vuxenutbildning, folkhögskola, vuxen, komvux, studieförbund, folkbildning, verksamhet, bidrag, landsbygd, statsbidrag, särskild, människa, kurs, resurs, glesbygd, yrkesvux, arbetslös, deltagare, studiecirkel, skogsbruk</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>1998/99 · Folkpartiet · GM02Ub425 · Flexiblare kursutbud i den högre utbildningen
-2010/11 · Moderaterna · GY02Ub312 · Antagning till högre utbildning
-2013/14 · Socialdemokraterna · H102Ub557 · Praktik på högskolans program
-1993/94 · Moderaterna · GH02Ub693 · Översyn av högskolelagen
-2005/06 · Folkpartiet · GT02Ub363 · Lektorer i gymnasieskolan</t>
+          <t>1989/90 · Miljöpartiet · GD02Ub293 · Nya studieförbund
+1990/91 · Socialdemokraterna · GE02Ub98 · med anledning av prop. 1990/91:82 Folkbildning
+1986/87 · Centerpartiet · GA02Ub247 · Folkhögskolan
+1990/91 · Folkpartiet · GE02Ub96 · med anledning av prop. 1990/91:82 Folkbildning
+1987/88 · Folkpartiet · GB02Ub352 · om folkhögskolorna</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -1580,16 +1580,16 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>stockholm, linköping, stiftelse, stockholmsregionen, beräknad, södertälje, trädgård, kommun, stat, norrköping, universitet, rut, legitimation, examensrätt, botanisk, verksamhet, hls, hantverkare, statlig, utrikes</t>
+          <t>örebro, barn, hörselskadad, ekeskola, synskadad, uf, hjälpmedel, rörelsehindrad, multifunktionshinder, resurscentrum, bemanning, rh, resurscent, svår, etikprövningsnämnd, jourskola, funkis, samordnare, bräcke, inkubator</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>1989/90 · Centerpartiet · GD02Ub663 · Stiftelsen Skånehantverk i Landskrona
-1988/89 · Folkpartiet · GC02Ub548 · Anslag till S:t Lukasstiftelsen
-1989/90 · Centerpartiet · GD02Ub674 · Botaniska trädgården i Göteborg
-1989/90 · Folkpartiet · GD02Ub563 · Göteborgs botaniska trädgård
-1987/88 · Folkpartiet · GB02Ub507 · om bidrag till S:t Lukasstiftelsens utbildningsverksamhet</t>
+          <t>1987/88 · Folkpartiet · GB02Ub289 · om Bräcke Östergård som nationellt kunskapscentrum
+1985/86 · Vänsterpartiet kommunisterna · G902ub273 · Ett resurscentrum för elever med rörelsehinder
+1988/89 · Folkpartiet · GC02Ub307 · Statligt stöd till handikappinstitutionen Bräcke Östergård
+1986/87 · Folkpartiet · GA02Ub347 · Utbildningen av svårt rörelsehindrade grundskoleelever
+2005/06 · Centerpartiet · GT02Ub241 · Nationell skolorganisation för hörselskadade</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
@@ -1616,24 +1616,24 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>förskola, barn, pedagogisk, verksamhet, barnomsorg, förälder, personal, behov, utveckling, lärande, fritidshem, förskollärare, kommun, kvalitet, omsorg, utveckla, arbeta, erbjuda, läroplan, förskoleklass</t>
+          <t>mobbning, barn, fysisk, idrott, ungdom, våld, aktivitet, hälsa, ung, körkort, vuxen, elev, fritid, arbete, rörelse, utsätta, mobba, aktiv, idrottshögskola, ansvar</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>1998/99 · Socialdemokraterna · GM02Ub229 · Utvecklingen av familjedaghem
-2010/11 · Socialdemokraterna · GY02Ub393 · En bra förskola för våra barn
-2008/09 · Socialdemokraterna · GW02Ub435 · En yrkeskategori i förskolan
-2008/09 · Socialdemokraterna · GW02Ub447 · Förskolan
-2005/06 · Socialdemokraterna · GT02Ub483 · Ungdomars rätt till en kvalitativ fritid</t>
+          <t>1987/88 · Folkpartiet · GB02Ub201 · om mobbning och våld i anslutning till skolarbetet
+1988/89 · Folkpartiet · GC02Ub207 · Mobbning och våld i skolan
+2014/15 · Moderaterna · H202586 · Rätten till skolidrott för barn med funktionsnedsättning
+2012/13 · Moderaterna · H002Ub420 · Skolidrott för barn med funktionsnedsättning
+1985/86 · Folkpartiet · G902ub296 · Mobbning i skolan</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -1976,24 +1976,24 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>student, förslag, studie, system, studerande, bidrag, högskola, studera, ekonomisk, studiemedel, enskild, csn, studiestöd, stat, regel, anslag, studiemedelssystem, särskild, betala, problem</t>
+          <t>land, svensk, kommun, ungdom, människa, språk, region, samhälle, län, utveckling, utveckla, funktionshind, kompetens, invandrare, stockholm, kunskap, område, plats, social, ekeskola</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2000/01 · Kristdemokraterna · GO02Ub412 · Nytt studiemedelssystem
-1999/2000 · Moderaterna · GN02Ub701 · Fribeloppsgränserna för studerande
-2003/04 · Folkpartiet · GR02Ub396 · Studiemedel
-2000/01 · Socialdemokraterna · GO02Ub720 · Dispensregler för CSN
-2002/03 · Folkpartiet · GQ02Ub262 · Flexibilitet i studiestödet</t>
+          <t>1998/99 · Socialdemokraterna · GM02Ub428 · Utländska akademiker
+1996/97 · Socialdemokraterna · GK02Ub212 · Översyn av svenska för invandrare
+1997/98 · Socialdemokraterna · GL02Ub417 · Glesbygdens utveckling och högskolornas roll
+2003/04 · Socialdemokraterna · GR02Ub447 · Utbildningsinsatser inom IT-området
+2002/03 · Socialdemokraterna · GQ02Ub240 · Arameiska</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -2016,24 +2016,24 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>elev, kommun, fristående, lärare, grundskola, skolverk, gymnasieskola, betyg, undervisning, nationell, kunskap, kommunal, förälder, mål, stöd, ämne, program, barn, ansvar, läsa</t>
+          <t>elev, lärare, kunskap, undervisning, grundskola, ämne, barn, mål, betyg, nationell, ansvar, ungdom, läsa, förälder, utveckla, nå, arbete, svensk, stöd, utveckling</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>1994/95 · Moderaterna · GI02Ub339 · Utvärdering inom skolan
-2001/02 · Centerpartiet · GP02Ub16 · med anledning av prop. 2001/02:35 Fristående skolor
-2004/05 · Kristdemokraterna · GS02Ub460 · Statens insatser för en likvärdig betygssättning
-1994/95 · Folkpartiet · GI02Ub7 · med anledning av prop. 1994/95:85 Betyg i det obligatoriska skolväsendet
-1994/95 · Kristen demokratisk samling · GI02Ub12 · med anledning av prop. 1994/95:85 Betyg i det obligatoriska skolväsendet</t>
+          <t>2000/01 · Moderaterna · GO02Ub206 · Skolplikt
+1997/98 · Moderaterna · GL02Ub2 · med anledning av prop. 1997/98:6 Förskoleklass och andra skollagsfrågor
+2000/01 · Vänsterpartiet · GO02Ub247 · Skolämnet idrott och hälsa
+1997/98 · Socialdemokraterna · GL02Ub4 · med anledning av prop. 1997/98:6 Förskoleklass och andra skollagsfrågor
+2000/01 · Moderaterna · GO02Ub311 · Idrott och hälsa på gymnasieskolan</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>KD</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -2056,24 +2056,24 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>barn, förskola, mobbning, förälder, elev, arbete, kommun, samhälle, ungdom, barnomsorg, människa, kunskap, verksamhet, ansvar, personal, problem, kvinna, lärare, ung, fysisk</t>
+          <t>lärare, lärarutbildning, kvinna, pedagogisk, kunskap, kompetens, yrke, läraryrke, krav, fortbildning, brist, läkare, arbete, personal, undervisning, rektor, utveckling, ämne, ansvar, utbildad</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>1997/98 · Moderaterna · GL02Ub202 · Mobbning
-1996/97 · Moderaterna · GK02Ub201 · Mobbning - ett folkhälsoproblem
-1998/99 · Kristdemokraterna · GM02Ub253 · Mobbning
-2004/05 · Kristdemokraterna · GS02Ub470 · Arbetet mot mobbning och sexuella trakasserier i skolan
-2002/03 · Vänsterpartiet · GQ02Ub556 · Sexualitet</t>
+          <t>2005/06 · Socialdemokraterna · GT02Ub269 · Högskoleutbildning av tandsköterskor
+2002/03 · Folkpartiet · GQ02Ub250 · Läraryrket
+2000/01 · Moderaterna · GO02Ub438 · Tandvårdsutbildning för tandsköterskor
+2001/02 · Folkpartiet · GP02Ub220 · Läraryrket
+2003/04 · Folkpartiet · GR02Ub417 · Uppvärdering av läraryrket</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -2096,24 +2096,24 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>forskning, universitet, högskola, svensk, forskarutbildning, anslag, utveckling, forskare, område, verksamhet, medel, resurs, internationell, förslag, samhälle, grundutbildning, kunskap, land, liten, vetenskaplig</t>
+          <t>kommun, fristående, elev, kommunal, skolverk, barn, friskola, verksamhet, förälder, förslag, välja, bidrag, grundskola, särskild, alternativ, stöd, undervisning, ekonomisk, kvalitet, nationell</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>1997/98 · Miljöpartiet · GL02Ub467 · Finanisiering av forskning och forskarutbildning
-1996/97 · Miljöpartiet · GK02Ub501 · Grundforskningsavdrag
-1994/95 · Miljöpartiet · GI02Ub662 · Grundforskning och forskarutbildning
-1998/99 · Miljöpartiet · GM02Ub455 · EU:s forskningsprogram och svensk forskning
-1997/98 · Miljöpartiet · GL02Ub469 · Svensk forskning och EU</t>
+          <t>1995/96 · Centerpartiet · GJ02Ub40 · med anledning av prop. 1995/96:200 Fristående skolor m.m.
+2003/04 · Kristdemokraterna · GR02Ub378 · Fristående skolor
+1997/98 · Centerpartiet · GL02Ub282 · Fristående skolor
+1994/95 · Centerpartiet · GI02Ub34 · med anledning av prop. 1994/95:157 Ändring av bidragsbestämmelserna för fristående skolor godkända för vanlig skolplikt m.m.
+1994/95 · Folkpartiet · GI02Ub31 · med anledning av prop. 1994/95:157 Ändring av bidragsbestämmelserna för fristående skolor godkända för vanlig skolplikt m.m.</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>gymnasieskola, kunskap, yrkesutbildning, företag, lärlingsutbildning, ungdom, program, arbetsliv, vuxenutbildning, kurs, lärande, arbetsmarknad, arbete, människa, kvalificerad, elev, samhälle, studie, krav, yrkeshögskola</t>
+          <t>högskola, forskning, universitet, utveckling, forskarutbildning, anslag, område, verksamhet, resurs, forskare, medel, svensk, grundutbildning, liten, internationell, utveckla, land, kvalitet, satsning, teknisk</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>1996/97 · Centerpartiet · GK02Ub219 · Lärlingsutbildning
-2005/06 · Folkpartiet · GT02Ub274 · Entreprenörskap på schemat
-1998/99 · Kristdemokraterna · GM02Ub234 · Ett heltäckande lärlingssystem
-2000/01 · Socialdemokraterna · GO02Ub329 · Gymnasieprogram för persontransporter
-2001/02 · Socialdemokraterna · GP02Ub378 · Gymnasieprogram för persontransporter</t>
+          <t>1999/2000 · Centerpartiet · GN02Ub27 · med anledning av prop. 1999/2000:81 Forskning för framtiden - en ny organisation för forskningsfinansiering
+1997/98 · Miljöpartiet · GL02Ub467 · Finanisiering av forskning och forskarutbildning
+2000/01 · Socialdemokraterna · GO02Ub517 · Mitthögskolan
+1998/99 · Socialdemokraterna · GM02Ub434 · Forskning vid Mitthögskolan
+1996/97 · Miljöpartiet · GK02Ub501 · Grundforskningsavdrag</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
@@ -2176,16 +2176,16 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>barn, funktionshind, språk, särskola, specialskola, ekeskola, undervisning, invandrare, land, svensk, läkare, vård, sfi, kompetens, medicinsk, brist, sjukdom, landsting, döv, stöd</t>
+          <t>gymnasieskola, elev, program, yrkesutbildning, kurs, kunskap, betyg, lärlingsutbildning, vuxenutbildning, företag, krav, arbetsliv, kvalificerad, lärande, individuell, gymnasium, högskola, förslag, kärnämne, gymnasieutbildning</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>2000/01 · Kristdemokraterna · GO02Ub422 · Behov av ökat antal neurologer
-1994/95 · Kristen demokratisk samling · GI02Ub345 · ANT-kunskap
-1998/99 · Socialdemokraterna · GM02Ub465 · Läkarutbildningen och Göteborg
-1997/98 · Kristdemokraterna · GL02Ub403 · ANT-kunskap
-2003/04 · Centerpartiet · GR02Ub301 · Ökad kunskap om smärta</t>
+          <t>1999/2000 · Kristdemokraterna · GN02Ub261 · Lärlingssystemet
+2002/03 · Kristdemokraterna · GQ02Ub342 · Försök med ny lärlingsutbildning i Småland
+1994/95 · Socialdemokraterna · GI02Ub381 · Riksgymnasierna för Rh-anpassad utbildning
+2004/05 · Moderaterna · GS02Ub294 · Hantverksutbildning
+2000/01 · Kristdemokraterna · GO02Ub323 · Lärlingssystem</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
@@ -2216,20 +2216,20 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>lärare, högskola, student, lärarutbildning, kvalitet, kunskap, pedagogisk, lärosäte, akademisk, universitet, krav, utveckla, kvinna, samhälle, kompetens, högskoleverk, undervisning, kurs, utveckling, arbete</t>
+          <t>student, högskola, studie, förslag, system, studerande, enskild, universitet, studera, lärosäte, studiemedel, ekonomisk, plats, kvalitet, social, människa, csn, problem, regel, studiestöd</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>1998/99 · Kristdemokraterna · GM02Ub458 · Jämställdhetsarbete i högskolan
-2004/05 · Socialdemokraterna · GS02Ub486 · Alternativa urval till högskolor
-1997/98 · Socialdemokraterna · GL02Ub415 · Uppdragsutbildning
-1999/2000 · Socialdemokraterna · GN02Ub487 · Jämställdhet i utbildningen
-2002/03 · Socialdemokraterna · GQ02Ub302 · Mentorskap och handledning för lärare</t>
+          <t>2001/02 · Vänsterpartiet · GP02Ub411 · Utbetalning av studiemedel
+1997/98 · Socialdemokraterna · GL02Ub702 · Fribeloppet i studiemedelssystemet
+2003/04 · Centerpartiet · GR02Ub339 · Studiemedel
+2001/02 · Socialdemokraterna · GP02Ub526 · Studiemedel och utbildningspoäng
+2000/01 · Moderaterna · GO02Ub705 · Studiestödsregler</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
@@ -2256,16 +2256,16 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>högskola, universitet, forskning, region, land, utveckling, plats, område, utveckla, län, stockholm, satsning, teknisk, verksamhet, resurs, göteborg, samarbete, bedriva, liten, regional</t>
+          <t>barn, förskola, mobbning, förälder, barnomsorg, arbete, verksamhet, samhälle, personal, elev, kommun, ansvar, problem, människa, kvinna, läroplan, våld, sexuell, flicka, vuxen</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>2001/02 · Centerpartiet · GP02Ub203 · Dalauniversitetet
-2000/01 · Centerpartiet · GO02Ub447 · Högskolan Dalarna som universitet
-2001/02 · Moderaterna · GP02Ub248 · Forskningsanslaget till Linköpings universitet
-2003/04 · Moderaterna · GR02Ub468 · Forskningsanslaget till Linköpings Universitet
-1994/95 · Centerpartiet · GI02Ub29 · med anledning av prop. 1994/95:139 Särskilda utbildningssatsningar inom högskolan</t>
+          <t>2001/02 · Kristdemokraterna · GP02Ub334 · Behovet av utbildning om barn och deras situation
+1999/2000 · Socialdemokraterna · GN02Ub39 · med anledning av prop. 1999/2000:123 Lämplighetsprövning av personal inom förskoleverksamhet, skola och skolbarnomsorg
+2003/04 · Kristdemokraterna · GR02Ub320 · Mobbning och våld
+2003/04 · Socialdemokraterna · GR02Ub479 · Lagstiftning mot mobbning
+2001/02 · Kristdemokraterna · GP02Ub304 · Mobbning</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>KD</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -2296,24 +2296,24 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>student, kommun, elev, fristående, kommunal, friskola, regel, välja, hög, ekonomisk, högskola, arbeta, fribelopp, studera, gymnasieskola, studiemedel, verksamhet, studie, körkort, införa</t>
+          <t>barn, förskola, förälder, kommun, barnomsorg, behov, personal, fritidshem, verksamhet, arbetstid, arbeta, erbjuda, pedagogisk, obekväm, kvalitet, arbete, utveckling, grupp, utveckla, förskollärare</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2010/11 · Moderaterna · GY02Ub416 · Fribeloppets avskaffande
-2007/08 · Moderaterna · GV02Ub339 · Skolskjuts oavsett skolform
-2006/07 · Moderaterna · GU02Ub329 · Avskaffande av fribeloppet
-2007/08 · Moderaterna · GV02Ub382 · Avskaffande av fribeloppet
-2007/08 · Moderaterna · GV02Ub377 · Fribeloppet</t>
+          <t>2006/07 · Kristdemokraterna · GU02Ub227 · Barns rätt till vila och rekreation
+2009/10 · Kristdemokraterna · GX02Ub491 · ”Nattis” och andra barnomsorgslösningar
+2008/09 · Socialdemokraterna · GW02Ub470 · Barnomsorg under obekväm arbetstid
+2013/14 · Miljöpartiet · H102Ub213 · Barnomsorg på obekväm arbetstid
+2007/08 · Socialdemokraterna · GV02Ub502 · Tidsgränser i barnomsorgen</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -2336,20 +2336,20 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>förskola, kommun, elev, barn, verksamhet, skollag, skolverk, lärare, pedagogisk, förslag, personal, kvalitet, fritidshem, huvudman, behov, lag, skolinspektion, krav, kommunal, enskild</t>
+          <t>elev, lärare, undervisning, kunskap, nationell, grundskola, ämne, mål, språk, betyg, utveckla, svensk, barn, skolverk, stöd, nå, pedagogisk, utveckling, resultat, lärarutbildning</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2008/09 · Socialdemokraterna · GW02Ub268 · Skolbibliotek och böcker
-2013/14 · Sverigedemokraterna · H102Ub13 · med anledning av prop. 2013/14:148 Vissa skollagsfrågor
-2007/08 · Socialdemokraterna · GV02Ub283 · En skola utan avgifter
-2013/14 · Vänsterpartiet · H102Ub11 · med anledning av prop. 2013/14:148 Vissa skollagsfrågor
-2009/10 · Socialdemokraterna · GX02Ub457 · Avgiftsfri skola</t>
+          <t>2008/09 · Socialdemokraterna · GW02Ub9 · med anledning av prop. 2008/09:66 En ny betygsskala
+2010/11 · Socialdemokraterna · GY02Ub2 · med anledning av prop. 2009/10:219 Betyg från årskurs 6 i grundskolan
+2008/09 · Socialdemokraterna · GW02Ub17 · med anledning av prop. 2008/09:87 Tydligare mål och kunskapskrav – nya läroplaner för skolan
+2011/12 · Sverigedemokraterna · GZ02Ub487 · Matematiksatsning i grundskolan
+2006/07 · Socialdemokraterna · GU02Ub377 · Nationella prov på modersmålet</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
@@ -2376,24 +2376,24 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>läkare, land, person, studie, vård, läkarutbildning, gammal, kunskap, patient, svensk, behov, sjukvård, landsting, lån, stipendium, brist, heltid, problem, ekonomisk, klinisk</t>
+          <t>land, svensk, kunskap, samhälle, människa, ungdom, person, läkare, kvinna, problem, ung, hälsa, gammal, behov, använda, vård, område, arbete, brist, rättighet</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2007/08 · Socialdemokraterna · GV02Ub275 · Utökad läkar- och tandläkarutbildning i Norrland
-2008/09 · Socialdemokraterna · GW02Ub211 · Utökad läkar- och tandläkarutbildning i Norrland
-2008/09 · Moderaterna · GW02Ub374 · Sjuksköterskor till läkarutbildning
-2008/09 · Moderaterna · GW02Ub352 · Allmäntjänstgöring för nyutexaminerade sjuksköterskor
-2009/10 · Moderaterna · GX02Ub331 · Allmäntjänstgöring för nyutexaminerade sjuksköterskor</t>
+          <t>2007/08 · Moderaterna · GV02Ub436 · Översyn av forskning på området integrativ medicin
+2006/07 · Socialdemokraterna · GU02Ub282 · Kvinnors sjukdomar
+2012/13 · Moderaterna · H002Ub333 · Behovet av geriatrik i utbildningen
+2006/07 · Folkpartiet · GU02Ub297 · Narkotikaupplysning
+2007/08 · Socialdemokraterna · GV02Ub560 · Behovet av läkare inom sjukvården</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -2416,20 +2416,20 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>ungdom, hälsa, fysisk, ung, barn, människa, aktivitet, mat, elev, idrott, psykisk, kunskap, problem, sjukdom, miljö, samhälle, ohälsa, arbete, liv, skolmat</t>
+          <t>ungdom, barn, fysisk, mat, elev, hälsa, kunskap, idrott, ung, grundskola, teckenspråk, skolmat, privatekonomi, ämne, lära, gymnasieskola, konsumentkunskap, gymnasium, lån, undervisning</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>2006/07 · Socialdemokraterna · GU02Ub342 · Skolans hälsoarbete
-2011/12 · Socialdemokraterna · GZ02Ub468 · Kondition och hälsa
-2008/09 · Moderaterna · GW02Ub234 · Fysisk aktivitet i skolan
-2007/08 · Moderaterna · GV02Ub237 · Den fysiska aktiviteten i skolan
-2008/09 · Socialdemokraterna · GW02Ub500 · Kunskap om mat</t>
+          <t>2010/11 · Kristdemokraterna · GY02Ub378 · Privatekonomi i gymnasieskolan
+2007/08 · Socialdemokraterna · GV02Ub296 · Hem- och konsumentkunskap
+2010/11 · Socialdemokraterna · GY02Ub316 · Hem- och konsumentkunskap även i gymnasiet
+2008/09 · Socialdemokraterna · GW02Ub228 · Hem- och konsumentkunskap
+2007/08 · Socialdemokraterna · GV02Ub501 · Hem- och konsumentkunskap i skolan</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
@@ -2456,24 +2456,24 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>elev, lärare, kunskap, undervisning, svensk, ämne, gymnasieskola, nationell, grundskola, språk, betyg, utveckla, mål, använda, program, lära, nå, resultat, utveckling, läsa</t>
+          <t>student, högskola, studie, hög, anslag, studiemedel, studera, förslag, höja, studerande, ekonomisk, fribelopp, kvalitet, universitet, arbeta, arbete, minska, plats, lärosäte, arbetsmarknad</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2008/09 · Vänsterpartiet · GW02Ub10 · med anledning av prop. 2008/09:66 En ny betygsskala
-2010/11 · Socialdemokraterna · GY02Ub2 · med anledning av prop. 2009/10:219 Betyg från årskurs 6 i grundskolan
-2010/11 · Moderaterna · GY02Ub331 · IT i skolan
-2008/09 · Moderaterna · GW02Ub310 · Undervisningsspråket i svensk grundskola
-2011/12 · Sverigedemokraterna · GZ02Ub487 · Matematiksatsning i grundskolan</t>
+          <t>2006/07 · Vänsterpartiet · GU02Ub333 · Utgiftsområde 15 Studiestöd
+2007/08 · Vänsterpartiet · GV02Ub478 · Utgiftsområde 15 Studiestöd
+2008/09 · Vänsterpartiet · GW02Ub454 · Utgiftsområde 15 Studiestöd
+2013/14 · Vänsterpartiet · H102Ub459 · Utgiftsområde 15 Studiestöd
+2011/12 · Moderaterna · GZ02Ub300 · Avskaffande av fribeloppet</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>V</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -2496,16 +2496,16 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>forskning, högskola, universitet, svensk, lärosäte, utveckling, hög, land, företag, internationell, område, utveckla, näringsliv, samhälle, kvalitet, kunskap, forskare, samarbete, student, nationell</t>
+          <t>gymnasieskola, arbetsmarknad, hög, behov, program, vuxenutbildning, ung, ungdom, kunskap, högskola, människa, jobb, yrkesutbildning, arbetsliv, arbete, företag, samhälle, gymnasium, läsa, kompetens</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>2012/13 · Socialdemokraterna · H002Ub440 · Mälardalens högskola
-2008/09 · Socialdemokraterna · GW02Ub1 · med anledning av prop. 2008/09:50 Ett lyft för forskning och innovation
-2008/09 · Socialdemokraterna · GW02Ub23 · med anledning av prop. 2008/09:134 Forskarutbildning med profilering och kvalitet
-2008/09 · Socialdemokraterna · GW02Ub24 · med anledning av prop. 2008/09:134 Forskarutbildning med profilering och kvalitet
-2012/13 · Socialdemokraterna · H002Ub418 · Forskning för att utveckla och miljöanpassa flyget</t>
+          <t>2008/09 · Socialdemokraterna · GW02Ub538 · Behovet av vuxenutbildning
+2007/08 · Socialdemokraterna · GV02Ub462 · Behovet av vuxenutbildning
+2007/08 · Socialdemokraterna · GV02Ub334 · Utbyggnad av högskolan
+2009/10 · Socialdemokraterna · GX02Ub353 · Korttidsutbildades rätt till ekonomisk ersättning
+2008/09 · Socialdemokraterna · GW02Ub326 · Vuxenstuderandes rätt till ekonomisk ersättning</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
@@ -2536,20 +2536,20 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>barn, förälder, förskola, barnomsorg, kommun, behov, kvinna, arbeta, personal, grupp, familj, samhälle, erbjuda, arbetstid, ungdom, liten, vuxen, land, utveckla, barngrupp</t>
+          <t>kommun, elev, fristående, kommunal, verksamhet, friskola, enskild, kostnad, skolverk, lag, huvudman, körkort, förslag, välja, skolinspektion, offentlig, skollag, regel, gymnasieskola, krav</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2006/07 · Socialdemokraterna · GU02Ub412 · Tidsgränser i förskolan
-2006/07 · Socialdemokraterna · GU02Ub413 · Avgiftsfri förskola
-2006/07 · Socialdemokraterna · GU02Ub389 · Den kommunala musikskolan
-2007/08 · Socialdemokraterna · GV02Ub256 · Musikskola för alla barn
-2008/09 · Socialdemokraterna · GW02Ub499 · Dolda skolavgifter</t>
+          <t>2006/07 · Moderaterna · GU02Ub298 · Ersättningen till fristående skolor
+2007/08 · Moderaterna · GV02Ub269 · Ersättning till fristående skolor
+2008/09 · Socialdemokraterna · GW02Ub399 · Ökat kommunalt inflytande vid etablering av friskolor
+2007/08 · Socialdemokraterna · GV02Ub283 · En skola utan avgifter
+2009/10 · Socialdemokraterna · GX02Ub278 · Ökat kommunalt inflytande vid etablering av friskolor</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
@@ -2576,20 +2576,20 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>arbetsmarknad, högskola, vuxenutbildning, behov, hög, arbete, jobb, studie, plats, människa, arbetsliv, yrkesutbildning, anslag, yrkeshögskola, studera, lärande, ung, ungdom, gymnasieskola, satsning</t>
+          <t>forskning, högskola, universitet, utveckling, svensk, lärosäte, hög, internationell, område, land, utveckla, forskare, kvalitet, näringsliv, samarbete, företag, samhälle, forskarutbildning, nationell, samverkan</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>2008/09 · Socialdemokraterna · GW02Ub538 · Behovet av vuxenutbildning
-2008/09 · Socialdemokraterna · GW02Ub256 · Studier för personer med låg utbildning
-2007/08 · Socialdemokraterna · GV02Ub462 · Behovet av vuxenutbildning
-2007/08 · Socialdemokraterna · GV02Ub409 · Studier för personer med låg utbildning
-2009/10 · Socialdemokraterna · GX02Ub353 · Korttidsutbildades rätt till ekonomisk ersättning</t>
+          <t>2008/09 · Socialdemokraterna · GW02Ub24 · med anledning av prop. 2008/09:134 Forskarutbildning med profilering och kvalitet
+2013/14 · Socialdemokraterna · H102Ub548 · Mälardalens högskola
+2007/08 · Kristdemokraterna · GV02Ub551 · Högskolan i Jönköping
+2008/09 · Socialdemokraterna · GW02Ub488 · Utbildning och forskning i Kalmar län
+2012/13 · Socialdemokraterna · H002Ub480 · Högskolan i Skövde</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
@@ -2616,16 +2616,16 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>barn, förskola, kommun, verksamhet, behov, kommunal, förälder, pedagogisk, fristående, förslag, personal, land, kvalitet, likvärdig, fritidshem, resurs, huvudman, hög, liten, svensk</t>
+          <t>lärare, svensk, undervisning, nationell, kunskap, grundskola, betyg, ämne, införa, hög, kvalitet, årskurs, stärka, behov, lärarutbildning, prov, resultat, stöd, läsa, skolverk</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2017/18 · Liberalerna · H502522 · Lärande förskola
-2019/20 · Liberalerna · H7023256 · En förskola för lärande
-2024/25 · Socialdemokraterna · HC021685 · Rätt till barnomsorg på obekväm arbetstid
-2020/21 · Socialdemokraterna · H8022083 · Jämlik förskola i hela landet
-2017/18 · Socialdemokraterna · H5021913 · Barnskötarlyft</t>
+          <t>2017/18 · Liberalerna · H5022555 · med anledning av prop. 2017/18:9 Skolstart vid sex års ålder
+2017/18 · Liberalerna · H502685 · med anledning av prop. 2017/18:14 Nationella prov - rättvisa, likvärdiga, digitala
+2018/19 · Moderaterna · H6022826 · Bättre kunskap om elevernas kunskaper
+2021/22 · Moderaterna · H9024275 · med anledning av prop. 2021/22:36 Ämnesbetyg – betygen ska bättre spegla elevers kunskaper
+2020/21 · Moderaterna · H8021704 · Stärkt koppling mellan slutbetyg och nationella prov i grundskolan</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -2656,24 +2656,24 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>student, studie, studera, studiemedel, arbetsmarknad, studerande, hög, person, yrkeshögskola, anslag, arbete, förslag, studiestöd, funktionsnedsättning, ekonomisk, högskola, stöd, människa, csn, arbeta</t>
+          <t>forskning, nivå, avancerad, grundnivå, högskola, forskarnivå, universitet, anslag, satsning, särskild, kunglig, stockholm, minska, teknisk, stöd, konstnärlig, förskola, statlig, verksamhet, bidrag</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>2016/17 · Moderaterna · H4023047 · Utgiftsområde 15 Studiestöd
-2016/17 · Kristdemokraterna · H4021532 · Utgiftsområde 15 Studiestöd
-2017/18 · Moderaterna · H5023856 · Utgiftsområde 15 Studiestöd
-2018/19 · Sverigedemokraterna · H6022374 · Utgiftsområde 15 Studiestöd
-2024/25 · Centerpartiet · HC022150 · Utgiftsområde 15 Studiestöd</t>
+          <t>2015/16 · Centerpartiet · H3023159 · Utgiftsområde 16 Utbildning och universitetsforskning
+2017/18 · Centerpartiet · H5023711 · Utgiftsområde 16 Utbildning och universitetsforskning
+2016/17 · Centerpartiet · H4023453 · Utgiftsområde 16 Utbildning och universitetsforskning
+2021/22 · Liberalerna · H9023994 · Utgiftsområde 16 Utbildning och universitetsforskning
+2021/22 · Vänsterpartiet · H9023272 · Utgiftsområde 16 Utbildning och universitetsforskning</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -2696,24 +2696,24 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>forskning, lärosäte, högskola, universitet, hög, forskare, student, kvalitet, land, innovation, svensk, anslag, akademisk, internationell, satsning, akademi, statlig, uppdrag, utveckling, nationell</t>
+          <t>forskning, lärosäte, hög, högskola, land, universitet, svensk, kvalitet, utveckling, student, forskare, stärka, behov, samhälle, internationell, satsning, område, innovation, nationell, utveckla</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>2014/15 · Kristdemokraterna · H2021046 · Full finansiering av läkarutbildningen i Örebro
-2016/17 · Kristdemokraterna · H402215 · Statlig finansiering av läkarutbildningen vid Örebro universitet
-2016/17 · Socialdemokraterna · H4021669 · Södertörns högskola
-2014/15 · Liberalerna · H202655 · Stärk läkarutbildningen vid Örebro universitet
-2021/22 · Centerpartiet · H9023207 · Likvärdig finansiering av läkarutbildningarna</t>
+          <t>2016/17 · Centerpartiet · H4023564 · med anledning av prop. 2016/17:50 Kunskap i samverkan - för samhällets utmaningar och stärkt konkurrenskraft
+2017/18 · Moderaterna · H5023407 · Life science och medtech
+2017/18 · Liberalerna · H5023041 · Forskning för mer kunskap och fler innovationer i Sverige
+2015/16 · Moderaterna · H3022772 · Forskning och innovation utvecklar Sverige
+2015/16 · Moderaterna · H3022452 · Life science</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>KD</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -2736,24 +2736,24 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>lärare, undervisning, ämne, svensk, nationell, betyg, grundskola, kunskap, lärarutbildning, prov, införa, årskurs, läsa, kvalitet, nyanländ, svenska, hög, sfi, resultat, stärka</t>
+          <t>anslag, studiemedel, studiestöd, förslag, skolbibliotek, studiestartsstöd, bidrag, csn, studielån, studie, minska, kostnad, satsning, teckenspråk, bibliotek, studera, stöd, höja, studerande, omställningsstudiestöd</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>2015/16 · Liberalerna · H3022766 · Karriärtjänster i utanförskapsområden
-2017/18 · Liberalerna · H5023040 · Nyanländas skolgång
-2014/15 · Kristdemokraterna · H2022006 · Låt nationella examinatorer rätta nationella prov
-2014/15 · Moderaterna · H2022758 · Mer idrott i skolan
-2014/15 · Moderaterna · H2022760 · Nationella prov</t>
+          <t>2017/18 · Centerpartiet · H5023702 · Utgiftsområde 15 Studiestöd
+2016/17 · Centerpartiet · H4023415 · Utgiftsområde 15 Studiestöd
+2021/22 · Moderaterna · H9024180 · Utgiftsområde 15 Studiestöd
+2018/19 · Centerpartiet · H6022636 · Utgiftsområde 15 Studiestöd
+2022/23 · Vänsterpartiet · HA021210 · Utgiftsområde 15 Studiestöd</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr"/>
@@ -2776,16 +2776,16 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>land, hög, svensk, företag, stärka, utveckling, arbetsmarknad, samhälle, kompetens, kunskap, utveckla, behov, jobb, ung, näringsliv, människa, arbete, tydlig, kvalitet, framtid</t>
+          <t>barn, förskola, kommun, förälder, verksamhet, stöd, behov, personal, pedagogisk, förslag, skolinspektion, huvudman, kommunal, fristående, lärare, skollag, fritidshem, ansvar, särskild, arbete</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2014/15 · Moderaterna · H202156 · Att satsa på entreprenörskap i skolan
-2018/19 · Centerpartiet · H6022850 · UF-företag och skolan
-2014/15 · Moderaterna · H2022011 · Ökad samverkan med aktörer som främjar entreprenörskap för unga
-2017/18 · Liberalerna · H5024192 · med anledning av skr. 2017/18:259 En strategi för svensk rymdverksamhet
-2015/16 · Sverigedemokraterna · H3023091 · Företagsamhet i skolan</t>
+          <t>2021/22 · Kristdemokraterna · H9024475 · med anledning av prop. 2021/22:132 Förskola för fler barn
+2017/18 · Vänsterpartiet · H5022341 · Fritidshem
+2015/16 · Moderaterna · H3021166 · Likabehandling av fristående skolor och förskolor
+2021/22 · Miljöpartiet · H9024589 · med anledning av prop. 2021/22:156 Resursskolor och tilläggsbelopp för särskilt stöd
+2021/22 · Moderaterna · H9024609 · med anledning av prop. 2021/22:156 Resursskolor och tilläggsbelopp för särskilt stöd</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
@@ -2816,24 +2816,24 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>barn, kvinna, samhälle, kunskap, svensk, ung, rättighet, människa, språk, förälder, religiös, undervisning, demokratisk, politisk, flicka, person, demokrati, kultur, land, lära</t>
+          <t>arbetsmarknad, student, jobb, studie, företag, person, ung, arbete, vuxenutbildning, sfi, hög, yrkeshögskola, studera, människa, kurs, arbeta, kunskap, ungdom, yrke, yrkesutbildning</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>2014/15 · Socialdemokraterna · H2021731 · Skolans ansvar för demokratin och allas lika värde
-2015/16 · Socialdemokraterna · H302834 · Motverkande av rasism och diskriminering i skolväsendet
-2015/16 · Socialdemokraterna · H302499 · Skolans ansvar för demokrati och mänskliga rättigheter
-2021/22 · Socialdemokraterna · H9021539 · Fördjupad MR- och demokratiutbildning i skolan
-2017/18 · Sverigedemokraterna · H5022298 · Könsmönster i läroplanen</t>
+          <t>2014/15 · Moderaterna · H2022275 · Fribeloppet för studerande
+2018/19 · Moderaterna · H6021449 · Omformat fribelopp
+2014/15 · Kristdemokraterna · H202861 · Slopat fribelopp för studiemedel
+2014/15 · Moderaterna · H2021217 · Förändring av inkomsttaket för studenter
+2015/16 · Sverigedemokraterna · H3021446 · Företagsdag på högstadiet och gymnasiet</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -2856,24 +2856,24 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>barn, lärare, stöd, rektor, skolinspektion, behov, arbete, undervisning, ansvar, skollag, psykisk, särskild, ung, åtgärd, kunskap, elevhälsa, tydlig, hälsa, uppdrag, trygghet</t>
+          <t>barn, ung, samhälle, kunskap, svensk, kvinna, undervisning, hälsa, människa, rättighet, våld, fysisk, arbete, lära, ungdom, flicka, kultur, läroplan, politisk, aktivitet</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2019/20 · Moderaterna · H7023094 · Trygghet och arbetsro för skolans medarbetare och elever
-2017/18 · Moderaterna · H5023355 · Kränkande behandling, frånvaro och psykisk ohälsa
-2015/16 · Moderaterna · H3021828 · Alla barns och elevers rätt att nå sin fulla potential
-2021/22 · Moderaterna · H9024613 · med anledning av prop. 2021/22:160 Skolans arbete med trygghet och studiero
-2019/20 · Liberalerna · H7023354 · Avveckla Skolinspektionens barn- och elevombud i sin nuvarande form</t>
+          <t>2025/26 · Kristdemokraterna · HD023098 · Skolsamlingar i kyrkan
+2014/15 · Socialdemokraterna · H2021731 · Skolans ansvar för demokratin och allas lika värde
+2015/16 · Socialdemokraterna · H302834 · Motverkande av rasism och diskriminering i skolväsendet
+2015/16 · Socialdemokraterna · H302499 · Skolans ansvar för demokrati och mänskliga rättigheter
+2024/25 · Kristdemokraterna · HC021135 · Skolavslutning med konfessionella inslag i kyrkan</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -2896,24 +2896,24 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>forskning, nivå, avancerad, grundnivå, högskola, forskarnivå, universitet, anslag, satsning, särskild, kunglig, minska, stockholm, teknisk, stöd, konstnärlig, verksamhet, bidrag, förskola, statlig</t>
+          <t>djurförsök, studium, djur, yrkesvägledning, försvar, totalförsvar, eu, metod, syv, militär, alternativ, krig, beredskap, svensk, ib, levande, handlingsplan, ukraina, ukrainsk, danmark</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>2017/18 · Centerpartiet · H5023711 · Utgiftsområde 16 Utbildning och universitetsforskning
-2016/17 · Centerpartiet · H4023453 · Utgiftsområde 16 Utbildning och universitetsforskning
-2015/16 · Centerpartiet · H3023159 · Utgiftsområde 16 Utbildning och universitetsforskning
-2021/22 · Liberalerna · H9023994 · Utgiftsområde 16 Utbildning och universitetsforskning
-2021/22 · Vänsterpartiet · H9023272 · Utgiftsområde 16 Utbildning och universitetsforskning</t>
+          <t>2020/21 · Moderaterna · H8023032 · Strategi för att fasa ut djurförsök
+2021/22 · Moderaterna · H9022089 · Utfasning av djurförsök
+2022/23 · Moderaterna · HA021088 · Utfasning av djurförsök
+2016/17 · Sverigedemokraterna · H4022600 · Totalförsvarskunskap i skolan
+2023/24 · Moderaterna · HB021280 · Utfasning av djurförsök</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>

</xml_diff>